<commit_message>
Add test suite - unit and integration tests
</commit_message>
<xml_diff>
--- a/dataAcquisition/Motec_MP/plottingRequest_BV_recreate.xlsx
+++ b/dataAcquisition/Motec_MP/plottingRequest_BV_recreate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SimEnv\dataAcquisition\Motec_MP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8010FCB-E134-4D37-AAB4-69D9A43D48CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DBD3B25-EE28-4A73-813C-F0DC569B168E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="1935" windowWidth="29040" windowHeight="15720" xr2:uid="{98CBB8D2-373D-4831-8E1A-176399598E12}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{98CBB8D2-373D-4831-8E1A-176399598E12}"/>
   </bookViews>
   <sheets>
     <sheet name="plotting" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1570" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1570" uniqueCount="196">
   <si>
     <t>mathFunction</t>
   </si>
@@ -437,9 +437,6 @@
     <t>timeseries_align</t>
   </si>
   <si>
-    <t>[244, 440]</t>
-  </si>
-  <si>
     <t>Fastest Lap Damper</t>
   </si>
   <si>
@@ -587,9 +584,6 @@
     <t>Inlet Manifold Pressure Mean [kPa]</t>
   </si>
   <si>
-    <t>[225, 300]</t>
-  </si>
-  <si>
     <t>Inlet Air Temp Sen Volt [V]</t>
   </si>
   <si>
@@ -612,6 +606,24 @@
   </si>
   <si>
     <t>global</t>
+  </si>
+  <si>
+    <t>[640, 720]</t>
+  </si>
+  <si>
+    <t>[235, 265]</t>
+  </si>
+  <si>
+    <t>Transmission Pressure Max [kPa]</t>
+  </si>
+  <si>
+    <t>Transmission Pressure Mean [kPa]</t>
+  </si>
+  <si>
+    <t>Coolant Pressure Max [kPa]</t>
+  </si>
+  <si>
+    <t>Coolant Pressure Mean [kPa]</t>
   </si>
 </sst>
 </file>
@@ -1202,25 +1214,25 @@
         <v>82</v>
       </c>
       <c r="V1" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="W1" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="Y1" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="X1" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="Z1" s="2" t="s">
-        <v>151</v>
-      </c>
       <c r="AA1" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="AB1" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="2" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1274,7 +1286,7 @@
         <v>89</v>
       </c>
       <c r="AB2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1329,12 +1341,12 @@
         <v>89</v>
       </c>
       <c r="AB3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>143</v>
+        <v>194</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>24</v>
@@ -1381,15 +1393,15 @@
         <v>31</v>
       </c>
       <c r="R4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="AB4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="5" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>144</v>
+        <v>195</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>24</v>
@@ -1436,15 +1448,15 @@
         <v>27</v>
       </c>
       <c r="R5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="AB5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>24</v>
@@ -1491,15 +1503,15 @@
         <v>23</v>
       </c>
       <c r="R6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="AB6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>24</v>
@@ -1546,15 +1558,15 @@
         <v>29</v>
       </c>
       <c r="R7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="AB7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
-        <v>141</v>
+        <v>192</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>24</v>
@@ -1601,15 +1613,15 @@
         <v>31</v>
       </c>
       <c r="R8" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="AB8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
-        <v>140</v>
+        <v>193</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>24</v>
@@ -1656,7 +1668,7 @@
         <v>27</v>
       </c>
       <c r="R9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="AB9" t="str">
         <f>AB8</f>
@@ -1712,10 +1724,10 @@
         <v>23</v>
       </c>
       <c r="R10" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="AB10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="11" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -1767,7 +1779,7 @@
         <v>29</v>
       </c>
       <c r="R11" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="AB11" t="str">
         <f t="shared" ref="AB11:AB48" si="1">AB10</f>
@@ -1823,7 +1835,7 @@
         <v>31</v>
       </c>
       <c r="R12" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="AB12" t="str">
         <f t="shared" si="1"/>
@@ -1879,7 +1891,7 @@
         <v>27</v>
       </c>
       <c r="R13" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="AB13" t="str">
         <f t="shared" si="1"/>
@@ -1938,7 +1950,7 @@
         <v>95</v>
       </c>
       <c r="AB14" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="15" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2111,7 +2123,7 @@
     </row>
     <row r="18" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="12" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B18" s="13" t="s">
         <v>24</v>
@@ -2158,7 +2170,7 @@
         <v>23</v>
       </c>
       <c r="R18" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="AB18" t="e">
         <f>#REF!</f>
@@ -2167,7 +2179,7 @@
     </row>
     <row r="19" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B19" s="13" t="s">
         <v>24</v>
@@ -2214,10 +2226,10 @@
         <v>29</v>
       </c>
       <c r="R19" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="AA19" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AB19" t="e">
         <f t="shared" si="1"/>
@@ -2276,13 +2288,13 @@
         <v>97</v>
       </c>
       <c r="R20" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="X20" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AB20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="21" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2337,7 +2349,7 @@
         <v>97</v>
       </c>
       <c r="R21" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="AB21" t="str">
         <f t="shared" si="1"/>
@@ -2396,7 +2408,7 @@
         <v>97</v>
       </c>
       <c r="R22" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="AB22" t="str">
         <f t="shared" si="1"/>
@@ -2455,7 +2467,7 @@
         <v>97</v>
       </c>
       <c r="R23" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="AB23" t="str">
         <f t="shared" si="1"/>
@@ -2511,10 +2523,10 @@
         <v>23</v>
       </c>
       <c r="R24" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AB24" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="25" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2566,7 +2578,7 @@
         <v>29</v>
       </c>
       <c r="R25" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AB25" t="str">
         <f t="shared" si="1"/>
@@ -2622,7 +2634,7 @@
         <v>31</v>
       </c>
       <c r="R26" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AB26" t="str">
         <f t="shared" si="1"/>
@@ -2678,7 +2690,7 @@
         <v>27</v>
       </c>
       <c r="R27" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AB27" t="str">
         <f t="shared" si="1"/>
@@ -2687,7 +2699,7 @@
     </row>
     <row r="28" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="16" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B28" s="16" t="s">
         <v>24</v>
@@ -2734,10 +2746,10 @@
         <v>23</v>
       </c>
       <c r="R28" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AB28" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="29" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2789,7 +2801,7 @@
         <v>29</v>
       </c>
       <c r="R29" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AB29" t="str">
         <f t="shared" si="1"/>
@@ -2845,10 +2857,10 @@
         <v>23</v>
       </c>
       <c r="R30" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AB30" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="31" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2900,7 +2912,7 @@
         <v>29</v>
       </c>
       <c r="R31" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AB31" t="str">
         <f t="shared" si="1"/>
@@ -2956,7 +2968,7 @@
         <v>31</v>
       </c>
       <c r="R32" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AB32" t="str">
         <f t="shared" si="1"/>
@@ -3012,7 +3024,7 @@
         <v>27</v>
       </c>
       <c r="R33" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AB33" t="str">
         <f t="shared" si="1"/>
@@ -3068,10 +3080,10 @@
         <v>23</v>
       </c>
       <c r="R34" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AB34" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="35" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3123,7 +3135,7 @@
         <v>29</v>
       </c>
       <c r="R35" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AB35" t="str">
         <f t="shared" si="1"/>
@@ -3179,7 +3191,7 @@
         <v>31</v>
       </c>
       <c r="R36" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AB36" t="str">
         <f t="shared" si="1"/>
@@ -3235,7 +3247,7 @@
         <v>27</v>
       </c>
       <c r="R37" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AB37" t="str">
         <f t="shared" si="1"/>
@@ -3291,10 +3303,10 @@
         <v>23</v>
       </c>
       <c r="R38" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AB38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="39" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3346,7 +3358,7 @@
         <v>29</v>
       </c>
       <c r="R39" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AB39" t="str">
         <f t="shared" si="1"/>
@@ -3402,7 +3414,7 @@
         <v>54</v>
       </c>
       <c r="R40" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AB40" t="str">
         <f t="shared" si="1"/>
@@ -3458,10 +3470,10 @@
         <v>23</v>
       </c>
       <c r="R41" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AB41" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="42" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3513,7 +3525,7 @@
         <v>29</v>
       </c>
       <c r="R42" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AB42" t="str">
         <f t="shared" si="1"/>
@@ -3569,10 +3581,10 @@
         <v>23</v>
       </c>
       <c r="R43" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="AB43" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="44" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3624,7 +3636,7 @@
         <v>29</v>
       </c>
       <c r="R44" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="AB44" t="str">
         <f t="shared" si="1"/>
@@ -3680,7 +3692,7 @@
         <v>54</v>
       </c>
       <c r="R45" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="AB45" t="str">
         <f t="shared" si="1"/>
@@ -3689,7 +3701,7 @@
     </row>
     <row r="46" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B46" s="23" t="s">
         <v>24</v>
@@ -3701,7 +3713,7 @@
         <v>9</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F46" s="23" t="s">
         <v>11</v>
@@ -3736,13 +3748,13 @@
         <v>23</v>
       </c>
       <c r="R46" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="AA46" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AB46" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="47" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3794,7 +3806,7 @@
         <v>29</v>
       </c>
       <c r="R47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="AB47" t="str">
         <f t="shared" si="1"/>
@@ -3803,7 +3815,7 @@
     </row>
     <row r="48" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B48" s="23" t="s">
         <v>24</v>
@@ -3850,7 +3862,7 @@
         <v>54</v>
       </c>
       <c r="R48" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AB48" t="str">
         <f t="shared" si="1"/>
@@ -3918,7 +3930,7 @@
         <v>4</v>
       </c>
       <c r="AB49" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="50" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3982,12 +3994,12 @@
         <v>4</v>
       </c>
       <c r="AB50" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="51" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>87</v>
@@ -4034,7 +4046,7 @@
         <v>31</v>
       </c>
       <c r="R51" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S51" t="b">
         <v>1</v>
@@ -4046,12 +4058,12 @@
         <v>4</v>
       </c>
       <c r="AB51" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="52" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>87</v>
@@ -4098,7 +4110,7 @@
         <v>27</v>
       </c>
       <c r="R52" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S52" t="b">
         <v>1</v>
@@ -4110,12 +4122,12 @@
         <v>4</v>
       </c>
       <c r="AB52" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="53" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B53" s="7" t="s">
         <v>87</v>
@@ -4162,7 +4174,7 @@
         <v>23</v>
       </c>
       <c r="R53" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S53" t="b">
         <v>1</v>
@@ -4174,12 +4186,12 @@
         <v>4</v>
       </c>
       <c r="AB53" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="54" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B54" s="7" t="s">
         <v>87</v>
@@ -4226,7 +4238,7 @@
         <v>29</v>
       </c>
       <c r="R54" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S54" t="b">
         <v>1</v>
@@ -4238,12 +4250,12 @@
         <v>4</v>
       </c>
       <c r="AB54" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="55" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B55" s="7" t="s">
         <v>87</v>
@@ -4290,7 +4302,7 @@
         <v>31</v>
       </c>
       <c r="R55" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="S55" t="b">
         <v>1</v>
@@ -4302,12 +4314,12 @@
         <v>4</v>
       </c>
       <c r="AB55" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="56" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B56" s="7" t="s">
         <v>87</v>
@@ -4354,7 +4366,7 @@
         <v>27</v>
       </c>
       <c r="R56" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="S56" t="b">
         <v>1</v>
@@ -4419,7 +4431,7 @@
         <v>23</v>
       </c>
       <c r="R57" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S57" t="b">
         <v>1</v>
@@ -4431,7 +4443,7 @@
         <v>4</v>
       </c>
       <c r="AB57" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="58" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4483,7 +4495,7 @@
         <v>29</v>
       </c>
       <c r="R58" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S58" t="b">
         <v>1</v>
@@ -4548,7 +4560,7 @@
         <v>31</v>
       </c>
       <c r="R59" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S59" t="b">
         <v>1</v>
@@ -4613,7 +4625,7 @@
         <v>27</v>
       </c>
       <c r="R60" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="S60" t="b">
         <v>1</v>
@@ -4690,7 +4702,7 @@
         <v>4</v>
       </c>
       <c r="AB61" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="62" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4890,7 +4902,7 @@
     </row>
     <row r="65" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="12" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B65" s="13" t="s">
         <v>87</v>
@@ -4949,12 +4961,12 @@
         <v>4</v>
       </c>
       <c r="AB65" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="66" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="12" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B66" s="13" t="s">
         <v>87</v>
@@ -5066,7 +5078,7 @@
         <v>23</v>
       </c>
       <c r="R67" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="S67" t="b">
         <v>1</v>
@@ -5078,10 +5090,10 @@
         <v>4</v>
       </c>
       <c r="V67" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="AB67" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="68" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5133,7 +5145,7 @@
         <v>29</v>
       </c>
       <c r="R68" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="S68" t="b">
         <v>1</v>
@@ -5145,7 +5157,7 @@
         <v>4</v>
       </c>
       <c r="V68" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="AB68" t="str">
         <f t="shared" si="2"/>
@@ -5201,7 +5213,7 @@
         <v>31</v>
       </c>
       <c r="R69" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="S69" t="b">
         <v>1</v>
@@ -5213,7 +5225,7 @@
         <v>4</v>
       </c>
       <c r="V69" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="AB69" t="str">
         <f t="shared" si="2"/>
@@ -5269,7 +5281,7 @@
         <v>27</v>
       </c>
       <c r="R70" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="S70" t="b">
         <v>1</v>
@@ -5281,7 +5293,7 @@
         <v>4</v>
       </c>
       <c r="V70" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="AB70" t="str">
         <f t="shared" si="2"/>
@@ -5337,7 +5349,7 @@
         <v>23</v>
       </c>
       <c r="R71" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="S71" t="b">
         <v>1</v>
@@ -5349,7 +5361,7 @@
         <v>4</v>
       </c>
       <c r="AB71" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="72" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5401,7 +5413,7 @@
         <v>29</v>
       </c>
       <c r="R72" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="S72" t="b">
         <v>1</v>
@@ -5466,7 +5478,7 @@
         <v>31</v>
       </c>
       <c r="R73" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="S73" t="b">
         <v>1</v>
@@ -5531,7 +5543,7 @@
         <v>27</v>
       </c>
       <c r="R74" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="S74" t="b">
         <v>1</v>
@@ -5549,7 +5561,7 @@
     </row>
     <row r="75" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="16" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B75" s="16" t="s">
         <v>87</v>
@@ -5596,7 +5608,7 @@
         <v>23</v>
       </c>
       <c r="R75" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="S75" t="b">
         <v>1</v>
@@ -5608,7 +5620,7 @@
         <v>4</v>
       </c>
       <c r="AB75" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="76" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5660,7 +5672,7 @@
         <v>29</v>
       </c>
       <c r="R76" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="S76" t="b">
         <v>1</v>
@@ -5725,7 +5737,7 @@
         <v>23</v>
       </c>
       <c r="R77" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="S77" t="b">
         <v>1</v>
@@ -5737,7 +5749,7 @@
         <v>4</v>
       </c>
       <c r="AB77" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="78" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5789,7 +5801,7 @@
         <v>29</v>
       </c>
       <c r="R78" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="S78" t="b">
         <v>1</v>
@@ -5854,7 +5866,7 @@
         <v>31</v>
       </c>
       <c r="R79" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="S79" t="b">
         <v>1</v>
@@ -5919,7 +5931,7 @@
         <v>27</v>
       </c>
       <c r="R80" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="S80" t="b">
         <v>1</v>
@@ -5984,7 +5996,7 @@
         <v>23</v>
       </c>
       <c r="R81" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="S81" t="b">
         <v>1</v>
@@ -5996,7 +6008,7 @@
         <v>4</v>
       </c>
       <c r="AB81" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="82" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6048,7 +6060,7 @@
         <v>29</v>
       </c>
       <c r="R82" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="S82" t="b">
         <v>1</v>
@@ -6113,7 +6125,7 @@
         <v>31</v>
       </c>
       <c r="R83" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="S83" t="b">
         <v>1</v>
@@ -6178,7 +6190,7 @@
         <v>27</v>
       </c>
       <c r="R84" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="S84" t="b">
         <v>1</v>
@@ -6243,7 +6255,7 @@
         <v>23</v>
       </c>
       <c r="R85" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="S85" t="b">
         <v>1</v>
@@ -6255,7 +6267,7 @@
         <v>4</v>
       </c>
       <c r="AB85" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="86" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6307,7 +6319,7 @@
         <v>29</v>
       </c>
       <c r="R86" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="S86" t="b">
         <v>1</v>
@@ -6372,7 +6384,7 @@
         <v>54</v>
       </c>
       <c r="R87" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="S87" t="b">
         <v>1</v>
@@ -6437,7 +6449,7 @@
         <v>23</v>
       </c>
       <c r="R88" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="S88" t="b">
         <v>1</v>
@@ -6449,7 +6461,7 @@
         <v>4</v>
       </c>
       <c r="AB88" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="89" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6501,7 +6513,7 @@
         <v>29</v>
       </c>
       <c r="R89" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="S89" t="b">
         <v>1</v>
@@ -6566,7 +6578,7 @@
         <v>23</v>
       </c>
       <c r="R90" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="S90" t="b">
         <v>1</v>
@@ -6578,7 +6590,7 @@
         <v>4</v>
       </c>
       <c r="AB90" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="91" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6630,7 +6642,7 @@
         <v>29</v>
       </c>
       <c r="R91" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="S91" t="b">
         <v>1</v>
@@ -6695,7 +6707,7 @@
         <v>54</v>
       </c>
       <c r="R92" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="S92" t="b">
         <v>1</v>
@@ -6713,7 +6725,7 @@
     </row>
     <row r="93" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="3" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B93" s="23" t="s">
         <v>87</v>
@@ -6725,7 +6737,7 @@
         <v>9</v>
       </c>
       <c r="E93" s="3" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F93" s="23" t="s">
         <v>11</v>
@@ -6760,7 +6772,7 @@
         <v>23</v>
       </c>
       <c r="R93" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="S93" t="b">
         <v>1</v>
@@ -6772,7 +6784,7 @@
         <v>4</v>
       </c>
       <c r="AB93" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="94" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -6824,7 +6836,7 @@
         <v>29</v>
       </c>
       <c r="R94" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="S94" t="b">
         <v>1</v>
@@ -6842,7 +6854,7 @@
     </row>
     <row r="95" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B95" s="23" t="s">
         <v>87</v>
@@ -6889,7 +6901,7 @@
         <v>54</v>
       </c>
       <c r="R95" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="S95" t="b">
         <v>1</v>
@@ -6956,7 +6968,7 @@
         <v>68</v>
       </c>
       <c r="R96" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="AB96" t="s">
         <v>65</v>
@@ -7011,7 +7023,7 @@
         <v>23</v>
       </c>
       <c r="R97" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="AB97" t="str">
         <f>A97</f>
@@ -7067,7 +7079,7 @@
         <v>23</v>
       </c>
       <c r="R98" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="S98" t="b">
         <v>1</v>
@@ -7079,13 +7091,13 @@
         <v>2</v>
       </c>
       <c r="AB98" t="str">
-        <f t="shared" ref="AB98:AB103" si="4">A98</f>
+        <f t="shared" ref="AB98:AB99" si="4">A98</f>
         <v>Falling Max Speed - Boxed</v>
       </c>
     </row>
     <row r="99" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="24" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B99" s="24" t="s">
         <v>87</v>
@@ -7112,7 +7124,7 @@
         <v>11</v>
       </c>
       <c r="J99" s="24" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K99" s="24" t="s">
         <v>11</v>
@@ -7132,7 +7144,7 @@
         <v>23</v>
       </c>
       <c r="R99" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="AB99" t="str">
         <f t="shared" si="4"/>
@@ -7193,13 +7205,13 @@
         <v>131</v>
       </c>
       <c r="X100" t="s">
-        <v>133</v>
+        <v>190</v>
       </c>
       <c r="Y100" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AB100" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="101" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -7256,13 +7268,13 @@
         <v>131</v>
       </c>
       <c r="X101" t="s">
-        <v>133</v>
+        <v>190</v>
       </c>
       <c r="Y101" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AB101" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="102" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -7319,18 +7331,18 @@
         <v>131</v>
       </c>
       <c r="X102" t="s">
-        <v>133</v>
+        <v>190</v>
       </c>
       <c r="Y102" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AB102" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="103" spans="1:28" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="25" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B103" s="25" t="s">
         <v>132</v>
@@ -7382,13 +7394,13 @@
         <v>131</v>
       </c>
       <c r="X103" t="s">
-        <v>133</v>
+        <v>190</v>
       </c>
       <c r="Y103" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AB103" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>